<commit_message>
Emparejar SE-28805 con el Multipress 3 Funciones de Black Series
Segunda de las tres filas que apuntaban a la maquina "de pie". Producto
confirma que el Press de Hombro y Pecho Dual de Pro Series (SE-28805) va
contra el Multipress 3 Funciones Black Series (BS-S5), no contra el
Pecho y Hombro de Pie Black Series (BS-S28).

La diferencia de precio no se mueve -BS-S5 y BS-S28 cuestan las dos
2.195 EUR-, asi que lo que se corrige es contra que maquina decimos que
competimos, no el numero. Con esto, tres de las cuatro gamas
(Elite, Black y Genesis) apuntan ya al Multipress; queda Advanced vs
Black RX, donde SE-28982 sigue con la de pie.

De paso esto libera BS-S28, que estaba en juego para PSE-28568.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKQ8SG8GjFdzRuTetWLx7y
</commit_message>
<xml_diff>
--- a/data/comparativa-titanium.xlsx
+++ b/data/comparativa-titanium.xlsx
@@ -2176,7 +2176,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Pecho y Hombro de Pie Black Series</t>
+          <t>Multipress 3 Funciones Black Series</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
@@ -2197,12 +2197,12 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>https://www.titaniumstrength.es/selectorizada-pecho-y-hombro-de-pie.html</t>
+          <t>https://www.titaniumstrength.es/titanium-strength-black-series-multipress-3-funciones.html</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Misma doble función, pero Titanium trabaja de pie</t>
+          <t>Cubre pecho y hombro, pero añade una tercera función y no es idéntica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Emparejar PSE-28568 con la Dual Pecho y Hombro de Pie de Elite
Estaba como "Sin equivalente" porque Black Series no tiene una dual que
haga las dos funciones. Producto aclara que el par existe, pero cruzando
de gama: "ellos la tienen en la elite y nosotros en la Pro Series". Asi
que la fila de Pro vs Black apunta a una maquina de Elite (EL-S28,
1.895 EUR) a proposito, y la observacion lo deja dicho para que nadie lo
tome por un error al revisarlo.

La equivalencia va como Directa: lo unico especial es la gama, la
maquina se corresponde una a una. Diego no llego a contestar a esa parte,
asi que sale de como lo explico; es una celda si hay que cambiarla.

Con el enlace puesto la fila deja de salir como "sin equivalente" en el
panel -build_titanium_comparison corta por ese campo antes que por nada
mas- y pasa a comparar: -196 EUR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKQ8SG8GjFdzRuTetWLx7y
</commit_message>
<xml_diff>
--- a/data/comparativa-titanium.xlsx
+++ b/data/comparativa-titanium.xlsx
@@ -1732,18 +1732,38 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Sin equivalente</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="7" t="n"/>
-      <c r="J2" s="8" t="n"/>
+          <t>Directa</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Dual Pecho y Hombro de Pie Elite Series</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>1895</v>
+      </c>
+      <c r="G2" s="4">
+        <f>C2-F2</f>
+        <v/>
+      </c>
+      <c r="H2" s="6">
+        <f>G2/F2</f>
+        <v/>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>https://www.titaniumstrength.es/selectorizada-dual-pecho-y-hombro-de-pie.html</t>
+        </is>
+      </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Black Series ofrece ambas funciones en máquinas separadas, no en una única dual equivalente</t>
+          <t>Caso especial: ellos la tienen en Elite y nosotros en Pro Series, por eso el par cruza de gama</t>
         </is>
       </c>
     </row>

</xml_diff>